<commit_message>
Print prompt and response
</commit_message>
<xml_diff>
--- a/data/output_marked.xlsx
+++ b/data/output_marked.xlsx
@@ -130,6 +130,21 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>AI_System</author>
+  </authors>
+  <commentList>
+    <comment ref="A3" authorId="0" shapeId="0">
+      <text>
+        <t>工资必须大于0，当前为0。</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -460,18 +475,17 @@
           <t>102</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>李四</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>工资必须大于 0</t>
-        </is>
+      <c r="C3" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>